<commit_message>
New features added to the solution
</commit_message>
<xml_diff>
--- a/config/Account_Booking.xlsx
+++ b/config/Account_Booking.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/natarajankanakasabapathy/FECTech/FDL-TestDataGeneration/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/natarajankanakasabapathy/FECTECH/FDL-TestDataGeneration/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DFFB99-F9FA-9845-8880-FD9A95D03E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EBFA2B8-2F24-E34C-A8DA-8C521925012B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4020" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{AC643E64-B35E-AD4D-A594-71A24CD144E3}"/>
+    <workbookView xWindow="-1460" yWindow="-21000" windowWidth="38400" windowHeight="21000" xr2:uid="{AC643E64-B35E-AD4D-A594-71A24CD144E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Columns" sheetId="1" r:id="rId1"/>
+    <sheet name="Tables" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Columns!$A$1:$AF$1</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="135">
   <si>
     <t>table_name</t>
   </si>
@@ -363,6 +364,87 @@
   </si>
   <si>
     <t>BBAN</t>
+  </si>
+  <si>
+    <t>table_kind</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>row_count</t>
+  </si>
+  <si>
+    <t>generation_mode</t>
+  </si>
+  <si>
+    <t>business_key_columns</t>
+  </si>
+  <si>
+    <t>primary_key_columns</t>
+  </si>
+  <si>
+    <t>partition_enabled</t>
+  </si>
+  <si>
+    <t>partition_columns</t>
+  </si>
+  <si>
+    <t>event_time_column</t>
+  </si>
+  <si>
+    <t>scd2_enabled</t>
+  </si>
+  <si>
+    <t>scd2_tracked_columns</t>
+  </si>
+  <si>
+    <t>delta_eligible</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>transactional</t>
+  </si>
+  <si>
+    <t>Account accounting entry table</t>
+  </si>
+  <si>
+    <t>snapshot</t>
+  </si>
+  <si>
+    <t>ACCT_ID;NTRY_SEQ_NB</t>
+  </si>
+  <si>
+    <t>Account accounting entry additional information</t>
+  </si>
+  <si>
+    <t>ACCT_ID;ACCT_CCY;NTRY_SEQ_NB</t>
+  </si>
+  <si>
+    <t>DF cash booking table</t>
+  </si>
+  <si>
+    <t>reference</t>
+  </si>
+  <si>
+    <t>Lookup mapping table</t>
+  </si>
+  <si>
+    <t>scd2_ready</t>
+  </si>
+  <si>
+    <t>Best initial SCD2 candidate</t>
+  </si>
+  <si>
+    <t>FX rates table</t>
+  </si>
+  <si>
+    <t>NL_IBAN</t>
   </si>
 </sst>
 </file>
@@ -939,7 +1021,9 @@
       <c r="F2" s="6"/>
       <c r="G2" s="4"/>
       <c r="H2" s="11"/>
-      <c r="I2" s="5"/>
+      <c r="I2" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
       <c r="L2" s="7"/>
@@ -3943,4 +4027,248 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A754C10-5D09-B046-AEAA-CE79D1764AFB}">
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M1" t="s">
+        <v>119</v>
+      </c>
+      <c r="N1" t="s">
+        <v>120</v>
+      </c>
+      <c r="O1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
+      </c>
+      <c r="E2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
+        <v>124</v>
+      </c>
+      <c r="F3" t="s">
+        <v>127</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+      <c r="E4" t="s">
+        <v>124</v>
+      </c>
+      <c r="F4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D5">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" t="s">
+        <v>106</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="s">
+        <v>93</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" t="s">
+        <v>103</v>
+      </c>
+      <c r="G6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>